<commit_message>
Add regenerated Excel report
</commit_message>
<xml_diff>
--- a/reports/ChangeManagement.xlsx
+++ b/reports/ChangeManagement.xlsx
@@ -413,30 +413,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Change ID</t>
+          <t>changeId</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>url</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>label</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CH05</t>
+          <t>CHG1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -446,347 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CHG01</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CH01</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CH03</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CH02</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CH04</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CH06</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CH09</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CH022</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CH024</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CH025</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CH07</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CH08</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CH010</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CH011</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>CHG02</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
           <t>APAC</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>CH012</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>CH023</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CHG1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>CH088</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>CH065</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>http://google.com</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>APAC</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TEST_LABEL</t>
         </is>
       </c>
     </row>

</xml_diff>